<commit_message>
Actualizo archivos .xlsx. No se deberian tener que commit pero me siguen apareciendo. Para mi porque son archivos modificados (es decir, estan en el repo)
</commit_message>
<xml_diff>
--- a/main_find_best_hyper/data/italia/df_best_mod.xlsx
+++ b/main_find_best_hyper/data/italia/df_best_mod.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:T28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,22 +556,22 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>(1306, 8)</t>
+          <t>(1254, 4)</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>(218, 8)</t>
+          <t>(209, 4)</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>(218, 8)</t>
+          <t>(209, 4)</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>['dt_vis', 'n_jug_aus_vis', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_edad_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_rat_jug_aus']</t>
+          <t>['dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_rat_jug_tit', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_aus']</t>
         </is>
       </c>
       <c r="N2" t="n">
@@ -584,20 +584,20 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 500, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l2', 'random_state': None, 'solver': 'saga', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 100, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'saga', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>48.57085346215781</v>
+        <v>51.00813008130082</v>
       </c>
       <c r="R2" t="n">
-        <v>44.23729418907818</v>
+        <v>43.90354539737523</v>
       </c>
       <c r="S2" t="n">
-        <v>54.6360153256705</v>
+        <v>54.72000000000001</v>
       </c>
       <c r="T2" t="n">
-        <v>55.04587155963303</v>
+        <v>57.89473684210527</v>
       </c>
     </row>
     <row r="3">
@@ -611,13 +611,9 @@
         <v>0.7</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>ml</t>
-        </is>
-      </c>
+        <v>0.2</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="b">
         <v>0</v>
@@ -630,22 +626,22 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>(3673, 8)</t>
+          <t>(525, 14)</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>(795, 8)</t>
+          <t>(88, 14)</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>(795, 8)</t>
+          <t>(88, 14)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>['dt_vis', 'n_jug_aus_vis', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_edad_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_rat_jug_aus']</t>
+          <t>['n_jug_aus_loc', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_faltas', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_valor_jug_aus']</t>
         </is>
       </c>
       <c r="N3" t="n">
@@ -653,25 +649,25 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>RandomForestClassifier</t>
+          <t>LogisticRegression</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 7, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 1, 'min_samples_split': 10, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 200, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 100, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'liblinear', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>47.67889387607697</v>
+        <v>52.1103896103896</v>
       </c>
       <c r="R3" t="n">
-        <v>42.74121994109512</v>
+        <v>50.86001204333791</v>
       </c>
       <c r="S3" t="n">
-        <v>53.70572207084469</v>
+        <v>56.38095238095239</v>
       </c>
       <c r="T3" t="n">
-        <v>55.34591194968554</v>
+        <v>57.95454545454546</v>
       </c>
     </row>
     <row r="4">
@@ -684,9 +680,7 @@
       <c r="C4" t="n">
         <v>0.7</v>
       </c>
-      <c r="D4" t="n">
-        <v>0.2</v>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="b">
@@ -700,22 +694,22 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>(147, 14)</t>
+          <t>(525, 27)</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>(25, 14)</t>
+          <t>(88, 27)</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>(25, 14)</t>
+          <t>(88, 27)</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>['dt_vis', 'n_jug_aus_vis', 'dif_prom_ult_part_dif_tarjetas_rojas', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_remates', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_edad_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_aus']</t>
+          <t>['temporada', 'es_copa', 'equipo_loc', 'equipo_vis', 'arbitro', 'cancha', 'dt_loc', 'dt_vis', 'n_jug_aus_loc', 'n_jug_aus_vis', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_faltas', 'dif_prom_ult_part_dif_remates', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_alt_jug_aus', 'dif_prom_valor_jug_aus']</t>
         </is>
       </c>
       <c r="N4" t="n">
@@ -723,25 +717,25 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>RandomForestClassifier</t>
+          <t>SVC</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 5, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 1, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 500, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+          <t>{'C': 5.0, 'break_ties': False, 'cache_size': 200, 'class_weight': None, 'coef0': 0.5, 'decision_function_shape': 'ovo', 'degree': 3, 'gamma': 'scale', 'kernel': 'poly', 'max_iter': -1, 'probability': False, 'random_state': None, 'shrinking': True, 'tol': 0.001, 'verbose': False}</t>
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>41.66666666666667</v>
+        <v>49.72222222222221</v>
       </c>
       <c r="R4" t="n">
-        <v>37.94162826420891</v>
+        <v>49.60001042318115</v>
       </c>
       <c r="S4" t="n">
-        <v>51.72413793103448</v>
+        <v>48.57142857142857</v>
       </c>
       <c r="T4" t="n">
-        <v>56.00000000000001</v>
+        <v>55.68181818181818</v>
       </c>
     </row>
     <row r="5">
@@ -752,16 +746,12 @@
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>ml</t>
-        </is>
-      </c>
+        <v>0.4</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="b">
         <v>0</v>
@@ -774,22 +764,22 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>(5023, 14)</t>
+          <t>(4507, 2)</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>(98, 14)</t>
+          <t>(751, 2)</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>(99, 14)</t>
+          <t>(752, 2)</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>['dt_vis', 'n_jug_aus_vis', 'dif_prom_ult_part_dif_tarjetas_rojas', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_remates', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_edad_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_aus']</t>
+          <t>['dif_prom_edad_jug_tit', 'dif_prom_rat_jug_tit']</t>
         </is>
       </c>
       <c r="N5" t="n">
@@ -797,25 +787,25 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>SVC</t>
+          <t>RandomForestClassifier</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>{'C': 5.0, 'break_ties': False, 'cache_size': 200, 'class_weight': None, 'coef0': 0.5, 'decision_function_shape': 'ovo', 'degree': 3, 'gamma': 'scale', 'kernel': 'poly', 'max_iter': -1, 'probability': False, 'random_state': None, 'shrinking': True, 'tol': 0.001, 'verbose': False}</t>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 3, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 4, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 200, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>51.3876608704195</v>
+        <v>46.60935044415871</v>
       </c>
       <c r="R5" t="n">
-        <v>48.71885596343801</v>
+        <v>40.72721074722166</v>
       </c>
       <c r="S5" t="n">
-        <v>53.78486055776892</v>
+        <v>54.49500554938957</v>
       </c>
       <c r="T5" t="n">
-        <v>64.64646464646465</v>
+        <v>55.85106382978723</v>
       </c>
     </row>
     <row r="6">
@@ -826,9 +816,11 @@
         <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D6" t="inlineStr"/>
+        <v>0.5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.2</v>
+      </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="b">
@@ -842,22 +834,22 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>(90, 25)</t>
+          <t>(574, 9)</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>(15, 25)</t>
+          <t>(96, 9)</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>(16, 25)</t>
+          <t>(96, 9)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>['equipo_loc', 'equipo_vis', 'arbitro', 'dt_loc', 'dt_vis', 'n_jug_aus_loc', 'n_jug_aus_vis', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_tarjetas_rojas', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_faltas', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_remates', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_tackles', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_alt_jug_aus', 'dif_prom_rat_jug_aus']</t>
+          <t>['n_jug_aus_loc', 'n_jug_aus_vis', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_faltas', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_edad_jug_aus']</t>
         </is>
       </c>
       <c r="N6" t="n">
@@ -865,25 +857,1531 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 7, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 4, 'min_samples_split': 10, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 100, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>54.52550452550452</v>
+      </c>
+      <c r="R6" t="n">
+        <v>48.99551320830813</v>
+      </c>
+      <c r="S6" t="n">
+        <v>50.35087719298246</v>
+      </c>
+      <c r="T6" t="n">
+        <v>54.16666666666666</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>(573, 21)</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>(96, 21)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>(96, 21)</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>['temporada', 'es_copa', 'equipo_loc', 'equipo_vis', 'arbitro', 'cancha', 'dt_loc', 'dt_vis', 'n_jug_aus_loc', 'n_jug_aus_vis', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_faltas', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_alt_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>5</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 3, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 4, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 200, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>48.97202561509943</v>
+      </c>
+      <c r="R7" t="n">
+        <v>40.52287581699346</v>
+      </c>
+      <c r="S7" t="n">
+        <v>53.33333333333334</v>
+      </c>
+      <c r="T7" t="n">
+        <v>53.125</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>30</v>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>(823, 17)</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>(137, 17)</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>(138, 17)</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>['n_jug_aus_loc', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_ataques_peligrosos', 'dif_prom_ult_part_dif_remates_fuera', 'dif_prom_ult_part_dif_pases_completados', 'dif_prom_ult_part_dif_remates_a_puerta', 'dif_prom_ult_part_dif_remates', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_puntos', 'dif_prom_edad_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_valor_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_sup', 'dif_prom_rat_jug_aus', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>SVC</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>{'C': 5.0, 'break_ties': False, 'cache_size': 200, 'class_weight': None, 'coef0': 1.0, 'decision_function_shape': 'ovo', 'degree': 5, 'gamma': 'scale', 'kernel': 'poly', 'max_iter': -1, 'probability': False, 'random_state': None, 'shrinking': True, 'tol': 0.001, 'verbose': False}</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>48.04687211934839</v>
+      </c>
+      <c r="R8" t="n">
+        <v>45.17373269166669</v>
+      </c>
+      <c r="S8" t="n">
+        <v>51.58536585365854</v>
+      </c>
+      <c r="T8" t="n">
+        <v>52.89855072463768</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>(327, 36)</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>(54, 36)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>(55, 36)</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>['temporada', 'equipo_loc', 'equipo_vis', 'arbitro', 'cancha', 'dt_vis', 'n_jug_aus_loc', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_ataques_peligrosos', 'dif_prom_ult_part_dif_faltas', 'dif_prom_ult_part_dif_remates_fuera', 'dif_prom_ult_part_dif_pases_completados', 'dif_prom_ult_part_dif_corneres', 'dif_prom_ult_part_dif_tiros_libres', 'dif_prom_ult_part_dif_remates_a_puerta', 'dif_prom_ult_part_dif_ataques', 'dif_prom_ult_part_dif_remates', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_puntos', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_remates_rechazados', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_valor_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_alt_jug_aus', 'dif_prom_rat_jug_aus', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>5</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 3, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 1, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 100, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>50.66666666666667</v>
+      </c>
+      <c r="R9" t="n">
+        <v>42.78367084538733</v>
+      </c>
+      <c r="S9" t="n">
+        <v>51.07692307692308</v>
+      </c>
+      <c r="T9" t="n">
+        <v>58.18181818181818</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>30</v>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>(327, 41)</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>(54, 41)</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>(55, 41)</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>['competicion', 'temporada', 'es_copa', 'equipo_loc', 'equipo_vis', 'arbitro', 'cancha', 'dt_loc', 'dt_vis', 'n_jug_aus_loc', 'n_jug_aus_vis', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_ataques_peligrosos', 'dif_prom_ult_part_dif_faltas', 'dif_prom_ult_part_dif_remates_fuera', 'dif_prom_ult_part_dif_pases_completados', 'dif_prom_ult_part_dif_corneres', 'dif_prom_ult_part_dif_tiros_libres', 'dif_prom_ult_part_dif_paradas', 'dif_prom_ult_part_dif_remates_a_puerta', 'dif_prom_ult_part_dif_ataques', 'dif_prom_ult_part_dif_remates', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_puntos', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_remates_rechazados', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_valor_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_alt_jug_aus', 'dif_prom_rat_jug_aus', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>5</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 7, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 1, 'min_samples_split': 10, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 100, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>49.33333333333334</v>
+      </c>
+      <c r="R10" t="n">
+        <v>48.57142857142857</v>
+      </c>
+      <c r="S10" t="n">
+        <v>49.84615384615385</v>
+      </c>
+      <c r="T10" t="n">
+        <v>52.72727272727272</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>45</v>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>(1254, 5)</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>(209, 5)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>(209, 5)</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>['dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_rat_jug_tit', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>5</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 3, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 1, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 200, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>45.10517799352751</v>
+      </c>
+      <c r="R11" t="n">
+        <v>40.23857019081586</v>
+      </c>
+      <c r="S11" t="n">
+        <v>55.27999999999999</v>
+      </c>
+      <c r="T11" t="n">
+        <v>55.02392344497608</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>45</v>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>(1154, 15)</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>(192, 15)</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>(193, 15)</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>['es_copa', 'n_jug_aus_loc', 'n_jug_aus_vis', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_remates_a_puerta', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>5</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>SVC</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'break_ties': False, 'cache_size': 200, 'class_weight': None, 'coef0': 1.0, 'decision_function_shape': 'ovo', 'degree': 3, 'gamma': 'scale', 'kernel': 'poly', 'max_iter': -1, 'probability': False, 'random_state': None, 'shrinking': True, 'tol': 0.001, 'verbose': False}</t>
+        </is>
+      </c>
+      <c r="Q12" t="n">
+        <v>46.11066559743384</v>
+      </c>
+      <c r="R12" t="n">
+        <v>39.95227231007264</v>
+      </c>
+      <c r="S12" t="n">
+        <v>54.95652173913044</v>
+      </c>
+      <c r="T12" t="n">
+        <v>53.8860103626943</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>45</v>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="b">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>(531, 27)</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>(89, 27)</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>(89, 27)</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>['temporada', 'es_copa', 'equipo_loc', 'equipo_vis', 'arbitro', 'cancha', 'dt_loc', 'dt_vis', 'n_jug_aus_loc', 'n_jug_aus_vis', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_remates_a_puerta', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_faltas', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_alt_jug_aus', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>5</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 3, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 4, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 100, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>50.9349593495935</v>
+      </c>
+      <c r="R13" t="n">
+        <v>42.58494530174599</v>
+      </c>
+      <c r="S13" t="n">
+        <v>55.09433962264151</v>
+      </c>
+      <c r="T13" t="n">
+        <v>55.0561797752809</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>45</v>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="b">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>(4507, 1)</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>(751, 1)</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>(752, 1)</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>['dif_prom_rat_jug_tit']</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>5</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
           <t>LogisticRegression</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>{'C': 5.0, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 100, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l2', 'random_state': None, 'solver': 'liblinear', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>48.56913299389738</v>
+      </c>
+      <c r="R14" t="n">
+        <v>42.03131067465102</v>
+      </c>
+      <c r="S14" t="n">
+        <v>55.64927857935627</v>
+      </c>
+      <c r="T14" t="n">
+        <v>56.64893617021277</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>45</v>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="b">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>(1538, 7)</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>(256, 7)</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>(257, 7)</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>['n_jug_aus_loc', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_faltas', 'dif_prom_edad_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup']</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>5</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
         <is>
           <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 100, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'saga', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
         </is>
       </c>
-      <c r="Q6" t="n">
-        <v>44.44444444444444</v>
-      </c>
-      <c r="R6" t="n">
-        <v>44.0422322775264</v>
-      </c>
-      <c r="S6" t="n">
-        <v>42.22222222222221</v>
-      </c>
-      <c r="T6" t="n">
-        <v>62.5</v>
+      <c r="Q15" t="n">
+        <v>47.35849056603774</v>
+      </c>
+      <c r="R15" t="n">
+        <v>41.03572862304296</v>
+      </c>
+      <c r="S15" t="n">
+        <v>56.15635179153095</v>
+      </c>
+      <c r="T15" t="n">
+        <v>54.86381322957199</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>45</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="b">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>(582, 21)</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>(97, 21)</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>(98, 21)</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>['temporada', 'es_copa', 'equipo_loc', 'equipo_vis', 'arbitro', 'cancha', 'dt_loc', 'dt_vis', 'n_jug_aus_loc', 'n_jug_aus_vis', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_faltas', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_alt_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>5</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 100, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'saga', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>56.36261673128033</v>
+      </c>
+      <c r="R16" t="n">
+        <v>48.53690387635341</v>
+      </c>
+      <c r="S16" t="n">
+        <v>50.17241379310344</v>
+      </c>
+      <c r="T16" t="n">
+        <v>58.16326530612245</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>45</v>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="b">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>(1239, 10)</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>(207, 10)</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>(207, 10)</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>['n_jug_aus_loc', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_puntos', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_rat_jug_tit', 'dif_prom_valor_jug_tit', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_sup', 'dif_prom_rat_jug_aus', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>5</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 100, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l1', 'random_state': None, 'solver': 'saga', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>47.25630560182418</v>
+      </c>
+      <c r="R17" t="n">
+        <v>42.86997529755221</v>
+      </c>
+      <c r="S17" t="n">
+        <v>54.17004048582996</v>
+      </c>
+      <c r="T17" t="n">
+        <v>51.69082125603865</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>45</v>
+      </c>
+      <c r="B18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="b">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>(327, 33)</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>(55, 33)</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>(55, 33)</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>['es_copa', 'arbitro', 'dt_vis', 'n_jug_aus_loc', 'n_jug_aus_vis', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_pases_completados', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_puntos', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_remates_a_puerta', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_remates_fuera', 'dif_prom_ult_part_dif_remates', 'dif_prom_ult_part_dif_remates_rechazados', 'dif_prom_ult_part_dif_tiros_libres', 'dif_prom_ult_part_dif_paradas', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_faltas', 'dif_prom_ult_part_dif_ataques_peligrosos', 'dif_prom_ult_part_dif_corneres', 'dif_prom_ult_part_dif_ataques', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_valor_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_sup', 'dif_prom_rat_jug_aus', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>5</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 3, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 4, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 200, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q18" t="n">
+        <v>43.46801346801346</v>
+      </c>
+      <c r="R18" t="n">
+        <v>40.24943310657596</v>
+      </c>
+      <c r="S18" t="n">
+        <v>52</v>
+      </c>
+      <c r="T18" t="n">
+        <v>47.27272727272727</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>45</v>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="b">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>(327, 41)</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>(55, 41)</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>(55, 41)</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>['competicion', 'temporada', 'es_copa', 'equipo_loc', 'equipo_vis', 'arbitro', 'cancha', 'dt_loc', 'dt_vis', 'n_jug_aus_loc', 'n_jug_aus_vis', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_pases_completados', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_puntos', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_remates_a_puerta', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_remates_fuera', 'dif_prom_ult_part_dif_remates', 'dif_prom_ult_part_dif_remates_rechazados', 'dif_prom_ult_part_dif_tiros_libres', 'dif_prom_ult_part_dif_paradas', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_faltas', 'dif_prom_ult_part_dif_ataques_peligrosos', 'dif_prom_ult_part_dif_corneres', 'dif_prom_ult_part_dif_ataques', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_valor_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_alt_jug_aus', 'dif_prom_rat_jug_aus', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>5</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 3, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 1, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 100, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>51.66666666666667</v>
+      </c>
+      <c r="R19" t="n">
+        <v>42.33100233100234</v>
+      </c>
+      <c r="S19" t="n">
+        <v>54.76923076923076</v>
+      </c>
+      <c r="T19" t="n">
+        <v>54.54545454545454</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>60</v>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="b">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>(1269, 4)</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>(211, 4)</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>(212, 4)</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>['dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_rat_jug_tit', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>5</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 3, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 4, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 100, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
+        <v>49.30499968235817</v>
+      </c>
+      <c r="R20" t="n">
+        <v>44.17700319710447</v>
+      </c>
+      <c r="S20" t="n">
+        <v>54.54545454545455</v>
+      </c>
+      <c r="T20" t="n">
+        <v>56.60377358490566</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>60</v>
+      </c>
+      <c r="B21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="b">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>(541, 19)</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>(90, 19)</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>(91, 19)</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>['temporada', 'cancha', 'dt_vis', 'n_jug_aus_loc', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_remates_a_puerta', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_faltas', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_alt_jug_aus', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>5</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 3, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 1, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 200, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
+        <v>56.12794612794612</v>
+      </c>
+      <c r="R21" t="n">
+        <v>48.45959595959595</v>
+      </c>
+      <c r="S21" t="n">
+        <v>52.40740740740741</v>
+      </c>
+      <c r="T21" t="n">
+        <v>63.73626373626373</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>60</v>
+      </c>
+      <c r="B22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="b">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>(541, 26)</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>(90, 26)</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>(91, 26)</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>['temporada', 'es_copa', 'equipo_loc', 'equipo_vis', 'arbitro', 'cancha', 'dt_loc', 'dt_vis', 'n_jug_aus_loc', 'n_jug_aus_vis', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_remates_a_puerta', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_faltas', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_alt_jug_aus', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>5</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 3, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 4, 'min_samples_split': 10, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 200, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
+        <v>52.7694654696943</v>
+      </c>
+      <c r="R22" t="n">
+        <v>46.81104569666386</v>
+      </c>
+      <c r="S22" t="n">
+        <v>51.85185185185185</v>
+      </c>
+      <c r="T22" t="n">
+        <v>60.43956043956044</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>60</v>
+      </c>
+      <c r="B23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="b">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>(4507, 1)</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>(751, 1)</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>(752, 1)</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>['dif_prom_rat_jug_tit']</t>
+        </is>
+      </c>
+      <c r="N23" t="n">
+        <v>5</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 3, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 4, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 200, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>47.23106620872922</v>
+      </c>
+      <c r="R23" t="n">
+        <v>41.46129713304789</v>
+      </c>
+      <c r="S23" t="n">
+        <v>54.82796892341842</v>
+      </c>
+      <c r="T23" t="n">
+        <v>56.64893617021277</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>60</v>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="b">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>(595, 9)</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>(99, 9)</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>(100, 9)</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>['n_jug_aus_loc', 'n_jug_aus_vis', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_faltas', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup']</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>5</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 100, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l2', 'random_state': None, 'solver': 'liblinear', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>49.47474747474747</v>
+      </c>
+      <c r="R24" t="n">
+        <v>43.85964912280702</v>
+      </c>
+      <c r="S24" t="n">
+        <v>54.28571428571429</v>
+      </c>
+      <c r="T24" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>60</v>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="b">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>(594, 21)</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>(99, 21)</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>(100, 21)</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>['temporada', 'es_copa', 'equipo_loc', 'equipo_vis', 'arbitro', 'cancha', 'dt_loc', 'dt_vis', 'n_jug_aus_loc', 'n_jug_aus_vis', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_faltas', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_alt_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>5</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>LogisticRegression</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>{'C': 0.1, 'class_weight': None, 'dual': False, 'fit_intercept': True, 'intercept_scaling': 1, 'l1_ratio': None, 'max_iter': 100, 'multi_class': 'auto', 'n_jobs': None, 'penalty': 'l2', 'random_state': None, 'solver': 'saga', 'tol': 0.0001, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>47.08374979177079</v>
+      </c>
+      <c r="R25" t="n">
+        <v>45.71940031326918</v>
+      </c>
+      <c r="S25" t="n">
+        <v>54.57627118644068</v>
+      </c>
+      <c r="T25" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>60</v>
+      </c>
+      <c r="B26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="b">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>(561, 20)</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>(93, 20)</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>(94, 20)</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>['arbitro', 'n_jug_aus_loc', 'dif_prom_ult_part_dif_pases_completados', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_puntos', 'dif_prom_ult_part_dif_remates_fuera', 'dif_prom_ult_part_dif_remates', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_ataques_peligrosos', 'dif_prom_ult_part_dif_corneres', 'dif_prom_edad_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_valor_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_sup', 'dif_prom_rat_jug_aus', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>5</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 7, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 4, 'min_samples_split': 10, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 100, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q26" t="n">
+        <v>46.41469641469642</v>
+      </c>
+      <c r="R26" t="n">
+        <v>42.96191984979171</v>
+      </c>
+      <c r="S26" t="n">
+        <v>52.85714285714285</v>
+      </c>
+      <c r="T26" t="n">
+        <v>48.93617021276596</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>60</v>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="b">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>(561, 29)</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>(93, 29)</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>(94, 29)</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>['temporada', 'equipo_loc', 'arbitro', 'dt_vis', 'n_jug_aus_loc', 'dif_prom_ult_part_dif_pases_completados', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_puntos', 'dif_prom_ult_part_dif_remates_a_puerta', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_remates_fuera', 'dif_prom_ult_part_dif_remates', 'dif_prom_ult_part_dif_tiros_libres', 'dif_prom_ult_part_dif_paradas', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_ataques_peligrosos', 'dif_prom_ult_part_dif_corneres', 'dif_prom_ult_part_dif_ataques', 'dif_prom_edad_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_valor_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_sup', 'dif_prom_alt_jug_aus', 'dif_prom_rat_jug_aus', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>5</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 7, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 1, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 200, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q27" t="n">
+        <v>60.20388325921605</v>
+      </c>
+      <c r="R27" t="n">
+        <v>58.56419163410044</v>
+      </c>
+      <c r="S27" t="n">
+        <v>54.28571428571429</v>
+      </c>
+      <c r="T27" t="n">
+        <v>62.76595744680851</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>60</v>
+      </c>
+      <c r="B28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="b">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>(338, 41)</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>(56, 41)</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>(57, 41)</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>['competicion', 'temporada', 'es_copa', 'equipo_loc', 'equipo_vis', 'arbitro', 'cancha', 'dt_loc', 'dt_vis', 'n_jug_aus_loc', 'n_jug_aus_vis', 'historial_entre_si_fecha', 'dif_prom_ult_part_dif_pases_completados', 'dif_prom_ult_part_dif_saques_de_banda', 'dif_prom_ult_part_dif_goles', 'dif_prom_ult_part_dif_puntos', 'dif_prom_ult_part_dif_tarjetas_amarillas', 'dif_prom_ult_part_dif_remates_a_puerta', 'dif_prom_ult_part_dif_posesion_de_balon', 'dif_prom_ult_part_dif_remates_fuera', 'dif_prom_ult_part_dif_remates', 'dif_prom_ult_part_dif_remates_rechazados', 'dif_prom_ult_part_dif_tiros_libres', 'dif_prom_ult_part_dif_paradas', 'dif_prom_ult_part_dif_fueras_de_juego', 'dif_prom_ult_part_dif_faltas', 'dif_prom_ult_part_dif_ataques_peligrosos', 'dif_prom_ult_part_dif_corneres', 'dif_prom_ult_part_dif_ataques', 'dif_prom_edad_jug_tit', 'dif_prom_alt_jug_tit', 'dif_prom_rat_jug_tit', 'dif_prom_valor_jug_tit', 'dif_prom_edad_jug_sup', 'dif_prom_alt_jug_sup', 'dif_prom_rat_jug_sup', 'dif_prom_valor_jug_sup', 'dif_prom_edad_jug_aus', 'dif_prom_alt_jug_aus', 'dif_prom_rat_jug_aus', 'dif_prom_valor_jug_aus']</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>5</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>RandomForestClassifier</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>{'bootstrap': True, 'ccp_alpha': 0.0, 'class_weight': None, 'criterion': 'entropy', 'max_depth': 3, 'max_features': 'auto', 'max_leaf_nodes': None, 'max_samples': None, 'min_impurity_decrease': 0.0, 'min_samples_leaf': 1, 'min_samples_split': 2, 'min_weight_fraction_leaf': 0.0, 'n_estimators': 200, 'n_jobs': None, 'oob_score': False, 'random_state': None, 'verbose': 0, 'warm_start': False}</t>
+        </is>
+      </c>
+      <c r="Q28" t="n">
+        <v>47.71062271062272</v>
+      </c>
+      <c r="R28" t="n">
+        <v>40.82125603864735</v>
+      </c>
+      <c r="S28" t="n">
+        <v>52.83582089552239</v>
+      </c>
+      <c r="T28" t="n">
+        <v>56.14035087719298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>